<commit_message>
added admin features and better ux.
</commit_message>
<xml_diff>
--- a/party-checkin/backend/responses.xlsx
+++ b/party-checkin/backend/responses.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="264">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="267">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -817,6 +817,15 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">EDUTSHU</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">rohit.m.sharma@ericsson.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Rohit Sharma</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">EZSHARO</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -913,8 +922,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:K75" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:K75"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:K76" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:K76"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Start time" dataDxfId="3"/>
@@ -3722,11 +3731,44 @@
         <x:v>17</x:v>
       </x:c>
     </x:row>
+    <x:row r="76" hidden="0">
+      <x:c r="A76">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B76" s="2">
+        <x:v>46210.4250810185</x:v>
+      </x:c>
+      <x:c r="C76" s="2">
+        <x:v>46210.4252893518</x:v>
+      </x:c>
+      <x:c r="D76" s="10" t="s">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="E76" s="10" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="F76" s="2"/>
+      <x:c r="G76" s="10" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="H76" s="10" t="s">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="I76" s="10" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J76" s="10" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="K76" s="10" t="s">
+        <x:v>30</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R0da17c8a2cc04800"/>
+    <x:tablePart r:id="R3f5a38929e0a47c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>